<commit_message>
test: strip Excel's local save path from the native fixture and re-pin
Removes only Excel's optional mc:AlternateContent/x15ac:absPath element
from xl/workbook.xml (privacy); the other 12 entries keep their raw
bytes, headers and order. Excel's original SHA-256 was
09104b6d0123eb53c9cd1a7ec900fce780d2c1520abc357f3049dc8631ede82c.
Against the edited file only the hash pin failed (8/9), so the edit
changed nothing the viewer reads; a new case asserts absPath is gone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-viewer/native-corner.xlsx
+++ b/tests/fixtures/xlsx-viewer/native-corner.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/julianshen/Library/Containers/com.microsoft.Excel/Data/Documents/officeview-native/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{914D3125-62EA-B842-9230-FCF7A292DD83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5480" yWindow="2320" windowWidth="27840" windowHeight="16820" xr2:uid="{3B88B68C-7640-E349-AC03-490814D7D8CE}"/>

</xml_diff>